<commit_message>
v10.18: Playwright Tests (3/6)
</commit_message>
<xml_diff>
--- a/PMS/tests/test-assets/user-list/partial_existing.xlsx
+++ b/PMS/tests/test-assets/user-list/partial_existing.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" dateCompatibility="false"/>
+  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="13">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -40,7 +40,7 @@
     <t xml:space="preserve">ingest1@uni.com</t>
   </si>
   <si>
-    <t xml:space="preserve">passwd</t>
+    <t xml:space="preserve">password</t>
   </si>
   <si>
     <t xml:space="preserve">student</t>
@@ -50,6 +50,15 @@
   </si>
   <si>
     <t xml:space="preserve">ingest4@uni.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ingest5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ingest5@uni.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">supervisor</t>
   </si>
 </sst>
 </file>
@@ -59,11 +68,12 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -79,6 +89,13 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -123,8 +140,16 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -251,55 +276,72 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16.13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16.12"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="1" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" s="1" t="s">
         <v>7</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D4" s="0" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B4" r:id="rId1" display="ingest5@uni.com"/>
+  </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>